<commit_message>
Modifying GUI and function combos to align with my plank
</commit_message>
<xml_diff>
--- a/Urchin Layouts.xlsx
+++ b/Urchin Layouts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhsch\Documents\Development\zmk-urchin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7BD340-D561-49C2-AD90-8A9BA5443A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D528A28-9A76-495D-8D8D-0580F95BBAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{4968A009-ADD2-40DC-B7CD-75D7443B6449}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4968A009-ADD2-40DC-B7CD-75D7443B6449}"/>
   </bookViews>
   <sheets>
     <sheet name="Layout" sheetId="9" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="201">
   <si>
     <t>esc</t>
   </si>
@@ -632,6 +632,15 @@
   </si>
   <si>
     <t xml:space="preserve">' </t>
+  </si>
+  <si>
+    <t>Set</t>
+  </si>
+  <si>
+    <t>BOOT</t>
+  </si>
+  <si>
+    <t>backspace</t>
   </si>
 </sst>
 </file>
@@ -1081,46 +1090,32 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
+      <right/>
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1131,7 +1126,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1321,15 +1316,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1337,11 +1323,23 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1695,45 +1693,45 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:42" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="72" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="N2" s="73" t="s">
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="72"/>
+      <c r="N2" s="72" t="s">
         <v>82</v>
       </c>
-      <c r="O2" s="73"/>
-      <c r="P2" s="73"/>
-      <c r="Q2" s="73"/>
-      <c r="R2" s="73"/>
-      <c r="S2" s="73"/>
-      <c r="T2" s="73"/>
-      <c r="U2" s="73"/>
-      <c r="V2" s="73"/>
-      <c r="W2" s="73"/>
-      <c r="X2" s="73"/>
-      <c r="Z2" s="73" t="s">
+      <c r="O2" s="72"/>
+      <c r="P2" s="72"/>
+      <c r="Q2" s="72"/>
+      <c r="R2" s="72"/>
+      <c r="S2" s="72"/>
+      <c r="T2" s="72"/>
+      <c r="U2" s="72"/>
+      <c r="V2" s="72"/>
+      <c r="W2" s="72"/>
+      <c r="X2" s="72"/>
+      <c r="Z2" s="72" t="s">
         <v>83</v>
       </c>
-      <c r="AA2" s="73"/>
-      <c r="AB2" s="73"/>
-      <c r="AC2" s="73"/>
-      <c r="AD2" s="73"/>
-      <c r="AE2" s="73"/>
-      <c r="AF2" s="73"/>
-      <c r="AG2" s="73"/>
-      <c r="AH2" s="73"/>
-      <c r="AI2" s="73"/>
-      <c r="AJ2" s="73"/>
+      <c r="AA2" s="72"/>
+      <c r="AB2" s="72"/>
+      <c r="AC2" s="72"/>
+      <c r="AD2" s="72"/>
+      <c r="AE2" s="72"/>
+      <c r="AF2" s="72"/>
+      <c r="AG2" s="72"/>
+      <c r="AH2" s="72"/>
+      <c r="AI2" s="72"/>
+      <c r="AJ2" s="72"/>
     </row>
     <row r="3" spans="2:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
@@ -2039,45 +2037,45 @@
       <c r="E7" s="22"/>
     </row>
     <row r="8" spans="2:42" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="73" t="s">
+      <c r="B8" s="72" t="s">
         <v>100</v>
       </c>
-      <c r="C8" s="73"/>
-      <c r="D8" s="73"/>
-      <c r="E8" s="73"/>
-      <c r="F8" s="73"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="73"/>
-      <c r="I8" s="73"/>
-      <c r="J8" s="73"/>
-      <c r="K8" s="73"/>
-      <c r="L8" s="73"/>
-      <c r="N8" s="73" t="s">
+      <c r="C8" s="72"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
+      <c r="I8" s="72"/>
+      <c r="J8" s="72"/>
+      <c r="K8" s="72"/>
+      <c r="L8" s="72"/>
+      <c r="N8" s="72" t="s">
         <v>84</v>
       </c>
-      <c r="O8" s="73"/>
-      <c r="P8" s="73"/>
-      <c r="Q8" s="73"/>
-      <c r="R8" s="73"/>
-      <c r="S8" s="73"/>
-      <c r="T8" s="73"/>
-      <c r="U8" s="73"/>
-      <c r="V8" s="73"/>
-      <c r="W8" s="73"/>
-      <c r="X8" s="73"/>
-      <c r="Z8" s="73" t="s">
+      <c r="O8" s="72"/>
+      <c r="P8" s="72"/>
+      <c r="Q8" s="72"/>
+      <c r="R8" s="72"/>
+      <c r="S8" s="72"/>
+      <c r="T8" s="72"/>
+      <c r="U8" s="72"/>
+      <c r="V8" s="72"/>
+      <c r="W8" s="72"/>
+      <c r="X8" s="72"/>
+      <c r="Z8" s="72" t="s">
         <v>101</v>
       </c>
-      <c r="AA8" s="73"/>
-      <c r="AB8" s="73"/>
-      <c r="AC8" s="73"/>
-      <c r="AD8" s="73"/>
-      <c r="AE8" s="73"/>
-      <c r="AF8" s="73"/>
-      <c r="AG8" s="73"/>
-      <c r="AH8" s="73"/>
-      <c r="AI8" s="73"/>
-      <c r="AJ8" s="73"/>
+      <c r="AA8" s="72"/>
+      <c r="AB8" s="72"/>
+      <c r="AC8" s="72"/>
+      <c r="AD8" s="72"/>
+      <c r="AE8" s="72"/>
+      <c r="AF8" s="72"/>
+      <c r="AG8" s="72"/>
+      <c r="AH8" s="72"/>
+      <c r="AI8" s="72"/>
+      <c r="AJ8" s="72"/>
     </row>
     <row r="9" spans="2:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="48" t="s">
@@ -2352,19 +2350,19 @@
       <c r="B15" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="N15" s="73" t="s">
+      <c r="N15" s="72" t="s">
         <v>81</v>
       </c>
-      <c r="O15" s="73"/>
-      <c r="P15" s="73"/>
-      <c r="Q15" s="73"/>
-      <c r="R15" s="73"/>
-      <c r="S15" s="73"/>
-      <c r="T15" s="73"/>
-      <c r="U15" s="73"/>
-      <c r="V15" s="73"/>
-      <c r="W15" s="73"/>
-      <c r="X15" s="73"/>
+      <c r="O15" s="72"/>
+      <c r="P15" s="72"/>
+      <c r="Q15" s="72"/>
+      <c r="R15" s="72"/>
+      <c r="S15" s="72"/>
+      <c r="T15" s="72"/>
+      <c r="U15" s="72"/>
+      <c r="V15" s="72"/>
+      <c r="W15" s="72"/>
+      <c r="X15" s="72"/>
       <c r="Z15"/>
       <c r="AA15"/>
       <c r="AB15"/>
@@ -2587,46 +2585,42 @@
   <dimension ref="A1:AI31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="51"/>
+    <col min="1" max="1" width="12.140625" style="51" customWidth="1"/>
     <col min="2" max="6" width="4.85546875" customWidth="1"/>
     <col min="10" max="21" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="71"/>
-      <c r="B1" s="72" t="s">
+      <c r="A1" s="68"/>
+      <c r="B1" s="69" t="s">
         <v>120</v>
       </c>
-      <c r="C1" s="72" t="s">
+      <c r="C1" s="69" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="72" t="s">
+      <c r="D1" s="69" t="s">
         <v>119</v>
       </c>
-      <c r="E1" s="72" t="s">
+      <c r="E1" s="69" t="s">
         <v>121</v>
       </c>
-      <c r="F1" s="72" t="s">
+      <c r="F1" s="69" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="68" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="72">
-        <v>2</v>
-      </c>
-      <c r="C2" s="72">
-        <v>2</v>
-      </c>
-      <c r="D2" s="72">
-        <v>2</v>
-      </c>
-      <c r="E2" s="72">
-        <v>2</v>
-      </c>
-      <c r="F2" s="72"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69">
+        <v>3</v>
+      </c>
+      <c r="E2" s="69">
+        <v>3</v>
+      </c>
+      <c r="F2" s="69"/>
       <c r="J2" s="10">
         <v>1</v>
       </c>
@@ -2661,20 +2655,20 @@
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A3" s="71" t="s">
+      <c r="A3" s="68" t="s">
         <v>96</v>
       </c>
-      <c r="B3" s="72">
+      <c r="B3" s="69">
         <v>2</v>
       </c>
-      <c r="C3" s="72">
+      <c r="C3" s="69">
         <v>2</v>
       </c>
-      <c r="D3" s="72"/>
-      <c r="E3" s="72">
+      <c r="D3" s="69"/>
+      <c r="E3" s="69">
         <v>2</v>
       </c>
-      <c r="F3" s="72"/>
+      <c r="F3" s="69"/>
       <c r="J3" s="10">
         <v>2</v>
       </c>
@@ -2733,20 +2727,20 @@
       </c>
     </row>
     <row r="4" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="71" t="s">
+      <c r="A4" s="68" t="s">
         <v>94</v>
       </c>
-      <c r="B4" s="72"/>
-      <c r="C4" s="72">
+      <c r="B4" s="69"/>
+      <c r="C4" s="69">
         <v>2</v>
       </c>
-      <c r="D4" s="72">
+      <c r="D4" s="69">
         <v>2</v>
       </c>
-      <c r="E4" s="72">
+      <c r="E4" s="69">
         <v>2</v>
       </c>
-      <c r="F4" s="72"/>
+      <c r="F4" s="69"/>
       <c r="J4" s="10">
         <v>3</v>
       </c>
@@ -2808,20 +2802,20 @@
       </c>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A5" s="71" t="s">
+      <c r="A5" s="68" t="s">
         <v>97</v>
       </c>
-      <c r="B5" s="72">
+      <c r="B5" s="69">
         <v>2</v>
       </c>
-      <c r="C5" s="72">
+      <c r="C5" s="69">
         <v>2</v>
       </c>
-      <c r="D5" s="72">
+      <c r="D5" s="69">
         <v>2</v>
       </c>
-      <c r="E5" s="72"/>
-      <c r="F5" s="72"/>
+      <c r="E5" s="69"/>
+      <c r="F5" s="69"/>
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
       <c r="L5" s="8"/>
@@ -2831,7 +2825,7 @@
       <c r="N5" s="55">
         <v>1</v>
       </c>
-      <c r="O5" s="70"/>
+      <c r="O5" s="67"/>
       <c r="P5" s="8"/>
       <c r="Q5" s="10">
         <v>1</v>
@@ -2871,18 +2865,18 @@
       </c>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A6" s="71" t="s">
+      <c r="A6" s="68" t="s">
         <v>191</v>
       </c>
-      <c r="B6" s="72">
+      <c r="B6" s="69">
         <v>1</v>
       </c>
-      <c r="C6" s="72">
+      <c r="C6" s="69">
         <v>1</v>
       </c>
-      <c r="D6" s="72"/>
-      <c r="E6" s="72"/>
-      <c r="F6" s="72"/>
+      <c r="D6" s="69"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="69"/>
       <c r="AA6" s="64" t="s">
         <v>124</v>
       </c>
@@ -2912,20 +2906,20 @@
       </c>
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A7" s="71" t="s">
+      <c r="A7" s="68" t="s">
         <v>192</v>
       </c>
-      <c r="B7" s="72"/>
-      <c r="C7" s="72">
+      <c r="B7" s="69"/>
+      <c r="C7" s="69">
         <v>2</v>
       </c>
-      <c r="D7" s="72">
+      <c r="D7" s="69">
         <v>2</v>
       </c>
-      <c r="E7" s="72">
+      <c r="E7" s="69">
         <v>5</v>
       </c>
-      <c r="F7" s="72"/>
+      <c r="F7" s="69"/>
       <c r="J7" t="s">
         <v>181</v>
       </c>
@@ -2958,18 +2952,18 @@
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A8" s="71" t="s">
+      <c r="A8" s="68" t="s">
         <v>99</v>
       </c>
-      <c r="B8" s="72"/>
-      <c r="C8" s="72"/>
-      <c r="D8" s="72">
+      <c r="B8" s="69"/>
+      <c r="C8" s="69"/>
+      <c r="D8" s="69">
         <v>1</v>
       </c>
-      <c r="E8" s="72">
+      <c r="E8" s="69">
         <v>1</v>
       </c>
-      <c r="F8" s="72"/>
+      <c r="F8" s="69"/>
       <c r="J8" s="10" t="s">
         <v>117</v>
       </c>
@@ -3031,6 +3025,18 @@
       </c>
     </row>
     <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A9" s="68" t="s">
+        <v>200</v>
+      </c>
+      <c r="B9" s="69">
+        <v>3</v>
+      </c>
+      <c r="C9" s="69">
+        <v>3</v>
+      </c>
+      <c r="D9" s="69"/>
+      <c r="E9" s="69"/>
+      <c r="F9" s="69"/>
       <c r="J9" s="10" t="s">
         <v>123</v>
       </c>
@@ -3158,10 +3164,14 @@
       <c r="N11" s="55" t="s">
         <v>98</v>
       </c>
-      <c r="O11" s="70"/>
+      <c r="O11" s="67"/>
       <c r="P11" s="8"/>
-      <c r="Q11" s="10"/>
-      <c r="R11" s="55"/>
+      <c r="Q11" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="R11" s="55" t="s">
+        <v>16</v>
+      </c>
       <c r="S11" s="8"/>
       <c r="T11" s="8"/>
       <c r="U11" s="8"/>
@@ -3442,7 +3452,7 @@
       <c r="L19" s="8"/>
       <c r="M19" s="55"/>
       <c r="N19" s="66"/>
-      <c r="O19" s="70"/>
+      <c r="O19" s="67"/>
       <c r="Q19" s="8"/>
       <c r="R19" s="8"/>
       <c r="S19" s="8"/>
@@ -3513,14 +3523,14 @@
       <c r="N22" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="Q22" s="67"/>
-      <c r="R22" s="68" t="s">
+      <c r="Q22" s="11"/>
+      <c r="R22" s="63" t="s">
         <v>66</v>
       </c>
-      <c r="S22" s="68" t="s">
+      <c r="S22" s="73" t="s">
         <v>65</v>
       </c>
-      <c r="T22" s="69" t="s">
+      <c r="T22" s="63" t="s">
         <v>64</v>
       </c>
       <c r="U22" s="59" t="s">
@@ -3538,7 +3548,7 @@
       <c r="AH22" s="51"/>
       <c r="AI22" s="51"/>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J23" s="10"/>
       <c r="K23" s="10">
         <v>6</v>
@@ -3552,14 +3562,14 @@
       <c r="N23" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="Q23" s="31"/>
-      <c r="R23" s="31" t="s">
+      <c r="Q23" s="10"/>
+      <c r="R23" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="S23" s="31" t="s">
+      <c r="S23" s="63" t="s">
         <v>62</v>
       </c>
-      <c r="T23" s="31" t="s">
+      <c r="T23" s="75" t="s">
         <v>61</v>
       </c>
       <c r="U23" s="10" t="s">
@@ -3591,14 +3601,11 @@
       <c r="N24" s="10">
         <v>0</v>
       </c>
-      <c r="O24" t="s">
-        <v>148</v>
-      </c>
       <c r="Q24" s="10"/>
       <c r="R24" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="S24" s="10" t="s">
+      <c r="S24" s="31" t="s">
         <v>59</v>
       </c>
       <c r="T24" s="10" t="s">
@@ -3626,8 +3633,11 @@
       <c r="M25" s="55" t="s">
         <v>76</v>
       </c>
-      <c r="N25" s="74" t="s">
+      <c r="N25" s="70" t="s">
         <v>14</v>
+      </c>
+      <c r="O25" t="s">
+        <v>148</v>
       </c>
       <c r="Q25" s="8"/>
       <c r="R25" s="8"/>
@@ -3663,6 +3673,9 @@
       <c r="J27" t="s">
         <v>186</v>
       </c>
+      <c r="Q27" t="s">
+        <v>198</v>
+      </c>
       <c r="AA27" s="64" t="s">
         <v>144</v>
       </c>
@@ -3719,7 +3732,7 @@
         <v>12</v>
       </c>
       <c r="M29" s="35" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="N29" s="10" t="s">
         <v>31</v>
@@ -3761,13 +3774,13 @@
         <v>16</v>
       </c>
       <c r="M30" s="35" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="N30" s="10" t="s">
         <v>15</v>
       </c>
       <c r="Q30" s="10" t="s">
-        <v>92</v>
+        <v>199</v>
       </c>
       <c r="R30" s="10"/>
       <c r="S30" s="10"/>
@@ -3789,7 +3802,7 @@
     </row>
     <row r="31" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A31" s="52"/>
-      <c r="J31" s="8"/>
+      <c r="J31" s="71"/>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
       <c r="M31" s="55"/>

</xml_diff>